<commit_message>
[monitoramento 14/09] Controle Semanal recebe a linha 12 (07-14/09)
22.192 impressoes e R$ 1.594,56 do console (set 7 - set 14); 123 cliques e
R$ 92,67 do export do Gerenciador; 5 pedidos e 8 unidades da bijecao com o
Business Report. Status VIGIA pela anomalia do L2025-T.

A nota declara as fontes mistas, a divergencia de 1 clique entre console e
export, a queda de impressoes como efeito das pausas da O5 em 09/09 e a
lacuna de serie em 01-06/09.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -115,6 +115,32 @@
   </si>
   <si>
     <t>Venda PXP 29/08 sem atribuição até 31/08. Auto L1618-o115/07 encontrada ativa (O4-006 não vigorou); pausada em 31/08. Atribuição de 29–31/08 ainda imatura."Geral DBA: ACOS de janela 83,9% (1 venda) → VIGIA; veredito do lance 0,48 na O5."</t>
+  </si>
+  <si>
+    <t>07/09/2026 a 14/09/2026</t>
+  </si>
+  <si>
+    <t>9.9 lido: Melhor Oferta 3 de 11 (R$ 1.196,21 / 7 un / 174 visualizações);
+Relâmpago 0 de 5 (19 visualizações) — falha de EXIBIÇÃO, não de conversão.
+Atribuição ao PREÇO DA OFERTA confirmada (5 pedidos, 3 SKUs, 4 campanhas).
+ACOS de 5,81% está inflado pela concentração de vendas com oferta — não
+recalibrar régua por ele. Participação de Ads de 86% é janela curta (6
+pedidos), não tendência; na Era da O5 era 38%. QUEDA DE IMPRESSÕES
+ESPERADA: 22.192 contra 47.770 em 24–31/08. É o efeito da O5 (4 campanhas
+pausadas em 09/09, no meio da janela), não colapso de entrega. CTR agregado
+SUBIU para 0,55% (era 0,41%) — entrega mais limpa, que era o objetivo.
+FONTES MISTAS: impressões e vendas do console (set 7–set 14); cliques e
+custo do export do Gerenciador, que veio com impressões zeradas. O console
+marca 122 cliques e o export 123 — diferença de 1, provável clique
+invalidado retroativamente. O custo não é exposto no painel do console.
+⚠️ L2025-T: 52 sessões (maior tráfego da semana), Melhor Oferta ativa, ZERO
+venda — era o motor de vendas (47 sessões / 4 un na Era). Vigiar na O6.
+Estado da O5 conferido: 12 ativas / 68 pausadas, nenhum zumbi. LACUNA DE
+SÉRIE: não há linha para 01–06/09 (o monitoramento de 07/09 foi eliminado
+pelo feriado) — a série não é contínua entre 31/08 e 14/09.</t>
+  </si>
+  <si>
+    <t>console Amazon Ads (set 7–set 14) + relatorios/amazon/monitoramento-14-09 + ciclos/Monitoramento-14-09.md</t>
   </si>
 </sst>
 </file>
@@ -125,7 +151,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -175,6 +201,12 @@
       <u/>
       <sz val="11"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -288,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -407,6 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -422,6 +455,7 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,6 +625,9 @@
                 <c:pt idx="5">
                   <c:v>46265</c:v>
                 </c:pt>
+                <c:pt idx="6">
+                  <c:v>46279</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -619,7 +656,7 @@
                   <c:v>0.46564023302817736</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>5.8116345574954847E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -779,11 +816,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1236001248"/>
-        <c:axId val="1236002880"/>
+        <c:axId val="-1413918016"/>
+        <c:axId val="-1413924000"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1236001248"/>
+        <c:axId val="-1413918016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -803,7 +840,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1236002880"/>
+        <c:crossAx val="-1413924000"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -811,7 +848,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1236002880"/>
+        <c:axId val="-1413924000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -831,7 +868,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1236001248"/>
+        <c:crossAx val="-1413918016"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1131,84 +1168,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="40"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
+      <c r="P1" s="41"/>
     </row>
     <row r="2" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
     </row>
     <row r="3" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="42"/>
-      <c r="N3" s="42"/>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="43"/>
+      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
     </row>
     <row r="4" spans="1:16" ht="21.95" customHeight="1">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44"/>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="45"/>
+      <c r="O4" s="45"/>
+      <c r="P4" s="45"/>
     </row>
     <row r="5" spans="1:16" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -1563,37 +1600,59 @@
       </c>
     </row>
     <row r="12" spans="1:16">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="12" t="str">
+      <c r="A12" s="40">
+        <v>46279</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="10">
+        <v>22192</v>
+      </c>
+      <c r="D12">
+        <v>123</v>
+      </c>
+      <c r="E12">
+        <v>92.67</v>
+      </c>
+      <c r="F12">
+        <v>1594.56</v>
+      </c>
+      <c r="G12">
+        <v>5</v>
+      </c>
+      <c r="H12">
+        <v>8</v>
+      </c>
+      <c r="I12" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="13" t="str">
+        <v>17.206863062479766</v>
+      </c>
+      <c r="J12" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="13" t="str">
+        <v>5.8116345574954847E-2</v>
+      </c>
+      <c r="K12" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L12" s="12" t="str">
+        <v>4.065040650406504E-2</v>
+      </c>
+      <c r="L12" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M12" s="14" t="str">
+        <v>0.75341463414634147</v>
+      </c>
+      <c r="M12" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N12" s="15"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="6"/>
+        <v>5.5425378514780098E-3</v>
+      </c>
+      <c r="N12" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O12" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="28"/>
@@ -3180,24 +3239,24 @@
       <c r="P60" s="9"/>
     </row>
     <row r="62" spans="1:16" ht="26.1" customHeight="1">
-      <c r="A62" s="43" t="s">
+      <c r="A62" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="43"/>
-      <c r="C62" s="43"/>
-      <c r="D62" s="43"/>
-      <c r="E62" s="43"/>
-      <c r="F62" s="43"/>
-      <c r="G62" s="43"/>
-      <c r="H62" s="43"/>
-      <c r="I62" s="43"/>
-      <c r="J62" s="43"/>
-      <c r="K62" s="43"/>
-      <c r="L62" s="43"/>
-      <c r="M62" s="43"/>
-      <c r="N62" s="43"/>
-      <c r="O62" s="43"/>
-      <c r="P62" s="43"/>
+      <c r="B62" s="44"/>
+      <c r="C62" s="44"/>
+      <c r="D62" s="44"/>
+      <c r="E62" s="44"/>
+      <c r="F62" s="44"/>
+      <c r="G62" s="44"/>
+      <c r="H62" s="44"/>
+      <c r="I62" s="44"/>
+      <c r="J62" s="44"/>
+      <c r="K62" s="44"/>
+      <c r="L62" s="44"/>
+      <c r="M62" s="44"/>
+      <c r="N62" s="44"/>
+      <c r="O62" s="44"/>
+      <c r="P62" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
[controle 21/09] Controle Semanal recebe a linha 13; GS1 segue em analise acima do prazo
Linha 13 (14-21/09) conferida: os 8 valores, status VIGIA, nota e fonte
batem com a proposta; formulas de I:M intactas; linha 14 limpa; exatamente
11 celulas alteradas (A:H e N:P).

GS1: documento reenviado em 15/09 ainda em analise em 21/09, quatro dias
uteis depois, acima do prazo de 1-2 dias do portal. Registrado no checklist
com a recomendacao de cobrar. Migracao de ASIN entra na O6 como NAO DECIDIR
AINDA.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Controle_Semanal" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="152511" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -141,6 +141,15 @@
   </si>
   <si>
     <t>console Amazon Ads (set 7–set 14) + relatorios/amazon/monitoramento-14-09 + ciclos/Monitoramento-14-09.md</t>
+  </si>
+  <si>
+    <t>14/09/2026 a 21/09/2026</t>
+  </si>
+  <si>
+    <t>SEM DIAGNÓSTICO — regra da véspera (MEMORIA 09/09): a O6 de 22/09 relê a Era 09–21/09 inteira. Esta linha é só registro. Primeira semana LIMPA pós-O5 (sem oferta): ACOS 17,4% com 2 vendas — P3070 R$ 616,18 (PI P3070, 15/09) e L2025-T R$ 132,90 (Geral, 15/09); bijeção console × Mestra fecha ao centav…</t>
+  </si>
+  <si>
+    <t>console Amazon Ads (set 14–set 21) + relatorios/amazon/monitoramento-21-09</t>
   </si>
 </sst>
 </file>
@@ -320,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -440,6 +449,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -455,12 +465,75 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE5E7EB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFECACA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF374151"/>
@@ -628,6 +701,9 @@
                 <c:pt idx="6">
                   <c:v>46279</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>46286</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -659,7 +735,7 @@
                   <c:v>5.8116345574954847E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.17428045068617504</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -816,11 +892,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-1413918016"/>
-        <c:axId val="-1413924000"/>
+        <c:axId val="-862632528"/>
+        <c:axId val="-862634704"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-1413918016"/>
+        <c:axId val="-862632528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -840,7 +916,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-1413924000"/>
+        <c:crossAx val="-862634704"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -848,7 +924,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-1413924000"/>
+        <c:axId val="-862634704"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -868,7 +944,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-1413918016"/>
+        <c:crossAx val="-862632528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1168,84 +1244,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="41"/>
-      <c r="P1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
     </row>
     <row r="2" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
     </row>
     <row r="3" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
-      <c r="O3" s="43"/>
-      <c r="P3" s="43"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
     </row>
     <row r="4" spans="1:16" ht="21.95" customHeight="1">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
-      <c r="O4" s="45"/>
-      <c r="P4" s="45"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="46"/>
     </row>
     <row r="5" spans="1:16" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -1618,10 +1694,10 @@
       <c r="F12">
         <v>1594.56</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="39">
         <v>5</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="39">
         <v>8</v>
       </c>
       <c r="I12" s="12">
@@ -1647,7 +1723,7 @@
       <c r="N12" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="O12" s="46" t="s">
+      <c r="O12" s="41" t="s">
         <v>33</v>
       </c>
       <c r="P12" t="s">
@@ -1655,37 +1731,59 @@
       </c>
     </row>
     <row r="13" spans="1:16">
-      <c r="A13" s="28"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="12" t="str">
+      <c r="A13" s="28">
+        <v>46286</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="10">
+        <v>43599</v>
+      </c>
+      <c r="D13" s="10">
+        <v>146</v>
+      </c>
+      <c r="E13" s="33">
+        <v>130.55000000000001</v>
+      </c>
+      <c r="F13" s="33">
+        <v>749.08</v>
+      </c>
+      <c r="G13" s="11">
+        <v>2</v>
+      </c>
+      <c r="H13" s="11">
+        <v>2</v>
+      </c>
+      <c r="I13" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="13" t="str">
+        <v>5.737878207583301</v>
+      </c>
+      <c r="J13" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="13" t="str">
+        <v>0.17428045068617504</v>
+      </c>
+      <c r="K13" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L13" s="12" t="str">
+        <v>1.3698630136986301E-2</v>
+      </c>
+      <c r="L13" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M13" s="14" t="str">
+        <v>0.89417808219178085</v>
+      </c>
+      <c r="M13" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N13" s="15"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="6"/>
+        <v>3.3487006582719786E-3</v>
+      </c>
+      <c r="N13" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O13" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="P13" s="47" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="28"/>
@@ -3239,24 +3337,24 @@
       <c r="P60" s="9"/>
     </row>
     <row r="62" spans="1:16" ht="26.1" customHeight="1">
-      <c r="A62" s="44" t="s">
+      <c r="A62" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="44"/>
-      <c r="C62" s="44"/>
-      <c r="D62" s="44"/>
-      <c r="E62" s="44"/>
-      <c r="F62" s="44"/>
-      <c r="G62" s="44"/>
-      <c r="H62" s="44"/>
-      <c r="I62" s="44"/>
-      <c r="J62" s="44"/>
-      <c r="K62" s="44"/>
-      <c r="L62" s="44"/>
-      <c r="M62" s="44"/>
-      <c r="N62" s="44"/>
-      <c r="O62" s="44"/>
-      <c r="P62" s="44"/>
+      <c r="B62" s="45"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
+      <c r="E62" s="45"/>
+      <c r="F62" s="45"/>
+      <c r="G62" s="45"/>
+      <c r="H62" s="45"/>
+      <c r="I62" s="45"/>
+      <c r="J62" s="45"/>
+      <c r="K62" s="45"/>
+      <c r="L62" s="45"/>
+      <c r="M62" s="45"/>
+      <c r="N62" s="45"/>
+      <c r="O62" s="45"/>
+      <c r="P62" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3267,22 +3365,22 @@
     <mergeCell ref="A4:P4"/>
   </mergeCells>
   <conditionalFormatting sqref="N6:N60">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>N6="NORMAL / AGUARDAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>N6="VIGIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>N6="INVESTIGAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>N6="PROBLEMA OPERACIONAL"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>N6="EMERGÊNCIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>N6="DADO INSUFICIENTE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[Monitoramento 28/09] Mestra corrigida e Controle linha 14 arquivados; lista do Prime Day de 28/09 (L2025-T e L1618-T entram, 5 seguem fora); vereditos EC-007..016 propostos; empilhamento oferta x promo de quantidade
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -150,6 +150,15 @@
   </si>
   <si>
     <t>console Amazon Ads (set 14–set 21) + relatorios/amazon/monitoramento-21-09</t>
+  </si>
+  <si>
+    <t>22/09/2026 a 28/09/2026</t>
+  </si>
+  <si>
+    <t>Primeira semana pós-O6 (10 ativas; SP-PP e EGC pausadas; loose da Geral a 0,45). ACOS 9,6% — 2 vendas, ambas na Geral: 3 un PXM R$ 580,08 (24/09, ES Capital) + 1 un L1618-T R$ 110,20, valorizadas A PREÇO COM DESCONTO — regra de atribuição do desconto no preço FIXADA (igual à Melhor Oferta; a promoçã…</t>
+  </si>
+  <si>
+    <t>console Amazon Ads (set 22–set 28) + relatorios/amazon/monitoramento-28-09</t>
   </si>
 </sst>
 </file>
@@ -450,6 +459,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -464,9 +476,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -704,6 +713,9 @@
                 <c:pt idx="7">
                   <c:v>46286</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>46293</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -738,7 +750,7 @@
                   <c:v>0.17428045068617504</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>9.5569913658225647E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -892,11 +904,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-862632528"/>
-        <c:axId val="-862634704"/>
+        <c:axId val="1054610720"/>
+        <c:axId val="1054618880"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-862632528"/>
+        <c:axId val="1054610720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -916,7 +928,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-862634704"/>
+        <c:crossAx val="1054618880"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -924,7 +936,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-862634704"/>
+        <c:axId val="1054618880"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -944,7 +956,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-862632528"/>
+        <c:crossAx val="1054610720"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1244,84 +1256,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
     </row>
     <row r="2" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
-      <c r="P2" s="43"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
     </row>
     <row r="3" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="45"/>
+      <c r="P3" s="45"/>
     </row>
     <row r="4" spans="1:16" ht="21.95" customHeight="1">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46"/>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="47"/>
+      <c r="O4" s="47"/>
+      <c r="P4" s="47"/>
     </row>
     <row r="5" spans="1:16" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -1685,13 +1697,13 @@
       <c r="C12" s="10">
         <v>22192</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="39">
         <v>123</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="39">
         <v>92.67</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="39">
         <v>1594.56</v>
       </c>
       <c r="G12" s="39">
@@ -1781,42 +1793,64 @@
       <c r="O13" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="P13" s="47" t="s">
+      <c r="P13" s="42" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:16">
-      <c r="A14" s="28"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="12" t="str">
+      <c r="A14" s="28">
+        <v>46293</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="10">
+        <v>19379</v>
+      </c>
+      <c r="D14" s="10">
+        <v>107</v>
+      </c>
+      <c r="E14" s="33">
+        <v>65.97</v>
+      </c>
+      <c r="F14" s="33">
+        <v>690.28</v>
+      </c>
+      <c r="G14" s="11">
+        <v>2</v>
+      </c>
+      <c r="H14" s="11">
+        <v>4</v>
+      </c>
+      <c r="I14" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="13" t="str">
+        <v>10.4635440351675</v>
+      </c>
+      <c r="J14" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="13" t="str">
+        <v>9.5569913658225647E-2</v>
+      </c>
+      <c r="K14" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L14" s="12" t="str">
+        <v>1.8691588785046728E-2</v>
+      </c>
+      <c r="L14" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M14" s="14" t="str">
+        <v>0.61654205607476631</v>
+      </c>
+      <c r="M14" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N14" s="15"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="6"/>
+        <v>5.5214407348160377E-3</v>
+      </c>
+      <c r="N14" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O14" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P14" s="42" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="28"/>
@@ -3337,24 +3371,24 @@
       <c r="P60" s="9"/>
     </row>
     <row r="62" spans="1:16" ht="26.1" customHeight="1">
-      <c r="A62" s="45" t="s">
+      <c r="A62" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="45"/>
-      <c r="C62" s="45"/>
-      <c r="D62" s="45"/>
-      <c r="E62" s="45"/>
-      <c r="F62" s="45"/>
-      <c r="G62" s="45"/>
-      <c r="H62" s="45"/>
-      <c r="I62" s="45"/>
-      <c r="J62" s="45"/>
-      <c r="K62" s="45"/>
-      <c r="L62" s="45"/>
-      <c r="M62" s="45"/>
-      <c r="N62" s="45"/>
-      <c r="O62" s="45"/>
-      <c r="P62" s="45"/>
+      <c r="B62" s="46"/>
+      <c r="C62" s="46"/>
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
+      <c r="F62" s="46"/>
+      <c r="G62" s="46"/>
+      <c r="H62" s="46"/>
+      <c r="I62" s="46"/>
+      <c r="J62" s="46"/>
+      <c r="K62" s="46"/>
+      <c r="L62" s="46"/>
+      <c r="M62" s="46"/>
+      <c r="N62" s="46"/>
+      <c r="O62" s="46"/>
+      <c r="P62" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
[05/10] Controle Semanal: linha 15 (29/09-05/10) conferida e subida; nota curta proposta para a coluna O
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>console Amazon Ads (set 22–set 28) + relatorios/amazon/monitoramento-28-09</t>
+  </si>
+  <si>
+    <t>29/09/2026 a 05/10/2026</t>
+  </si>
+  <si>
+    <t>Semana de preço limpo + 1º dia do Prime Day. 6 compras/9 un: Geral 4 (P4080 1ª venda, P3060 ×2, L1618-B, L1623-T), PI P3070 1 (alvo B0CTMZHJFJ), PI PXM 1 (3 un). ACOS 3,1% — n pequeno, não é base de escala. Prime Day às 15h de 05/10: Melhor Oferta PXP "Apresenta problemas" (preço promocional ≠ preço…</t>
+  </si>
+  <si>
+    <t>relatorios/amazon/monitoramento-05-10/ (export, BR 29/09–04/10, prints) + ciclos/Monitoramento-05-10.md</t>
   </si>
 </sst>
 </file>
@@ -716,6 +725,9 @@
                 <c:pt idx="8">
                   <c:v>46293</c:v>
                 </c:pt>
+                <c:pt idx="9">
+                  <c:v>46300</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -753,7 +765,7 @@
                   <c:v>9.5569913658225647E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>3.0904064203445228E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -904,11 +916,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1054610720"/>
-        <c:axId val="1054618880"/>
+        <c:axId val="360762896"/>
+        <c:axId val="360770512"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1054610720"/>
+        <c:axId val="360762896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -928,7 +940,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1054618880"/>
+        <c:crossAx val="360770512"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -936,7 +948,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1054618880"/>
+        <c:axId val="360770512"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -956,7 +968,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1054610720"/>
+        <c:crossAx val="360762896"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1853,37 +1865,59 @@
       </c>
     </row>
     <row r="15" spans="1:16">
-      <c r="A15" s="28"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="12" t="str">
+      <c r="A15" s="28">
+        <v>46300</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="10">
+        <v>39236</v>
+      </c>
+      <c r="D15" s="10">
+        <v>125</v>
+      </c>
+      <c r="E15" s="33">
+        <v>110.44</v>
+      </c>
+      <c r="F15" s="33">
+        <v>3573.64</v>
+      </c>
+      <c r="G15" s="11">
+        <v>6</v>
+      </c>
+      <c r="H15" s="11">
+        <v>9</v>
+      </c>
+      <c r="I15" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="13" t="str">
+        <v>32.358203549438606</v>
+      </c>
+      <c r="J15" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="13" t="str">
+        <v>3.0904064203445228E-2</v>
+      </c>
+      <c r="K15" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L15" s="12" t="str">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="L15" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M15" s="14" t="str">
+        <v>0.88351999999999997</v>
+      </c>
+      <c r="M15" s="14">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N15" s="15"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="6"/>
+        <v>3.185849729839943E-3</v>
+      </c>
+      <c r="N15" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O15" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="P15" s="42" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="28"/>

</xml_diff>

<commit_message>
[13/10] Controle Semanal: linha 16 (06-12/10) conferida e subida; status, nota e fonte a preencher
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>relatorios/amazon/monitoramento-05-10/ (export, BR 29/09–04/10, prints) + ciclos/Monitoramento-05-10.md</t>
+  </si>
+  <si>
+    <t>06/10/2026 a 12/10/2026</t>
   </si>
 </sst>
 </file>
@@ -490,68 +493,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE5E7EB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFECACA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF374151"/>
@@ -646,7 +588,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -728,6 +669,9 @@
                 <c:pt idx="9">
                   <c:v>46300</c:v>
                 </c:pt>
+                <c:pt idx="10">
+                  <c:v>46307</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -768,7 +712,7 @@
                   <c:v>3.0904064203445228E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>8.3921738671854401E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -916,11 +860,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="360762896"/>
-        <c:axId val="360770512"/>
+        <c:axId val="1962862624"/>
+        <c:axId val="1962858816"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="360762896"/>
+        <c:axId val="1962862624"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -940,7 +884,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="360770512"/>
+        <c:crossAx val="1962858816"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -948,7 +892,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="360770512"/>
+        <c:axId val="1962858816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -968,7 +912,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="360762896"/>
+        <c:crossAx val="1962862624"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1920,33 +1864,49 @@
       </c>
     </row>
     <row r="16" spans="1:16">
-      <c r="A16" s="28"/>
-      <c r="B16" s="36"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="12" t="str">
+      <c r="A16" s="28">
+        <v>46307</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="10">
+        <v>39389</v>
+      </c>
+      <c r="D16" s="10">
+        <v>189</v>
+      </c>
+      <c r="E16" s="33">
+        <v>143.22</v>
+      </c>
+      <c r="F16" s="33">
+        <v>1706.59</v>
+      </c>
+      <c r="G16" s="11">
+        <v>7</v>
+      </c>
+      <c r="H16" s="11">
+        <v>12</v>
+      </c>
+      <c r="I16" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="13" t="str">
+        <v>11.915863706186286</v>
+      </c>
+      <c r="J16" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="13" t="str">
+        <v>8.3921738671854401E-2</v>
+      </c>
+      <c r="K16" s="13">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L16" s="12" t="str">
+        <v>3.7037037037037035E-2</v>
+      </c>
+      <c r="L16" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M16" s="14" t="str">
+        <v>0.75777777777777777</v>
+      </c>
+      <c r="M16" s="14">
         <f t="shared" si="4"/>
-        <v/>
+        <v>4.7982939399324681E-3</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="1"/>
@@ -3433,22 +3393,22 @@
     <mergeCell ref="A4:P4"/>
   </mergeCells>
   <conditionalFormatting sqref="N6:N60">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>N6="NORMAL / AGUARDAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>N6="VIGIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>N6="INVESTIGAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>N6="PROBLEMA OPERACIONAL"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>N6="EMERGÊNCIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="0" priority="6">
       <formula>N6="DADO INSUFICIENTE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[19/10] vigias: exata "pia de cozinha" da 6B disparou (32 cli vit / 0) -> EC-021 pausar alvo proposta; PI P3070 sem alvo na regua, P3070 15/10 organico; Controle linha 17 colada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
+++ b/dados/Controle_Semanal_Amazon_Ads_Winnet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t>CONTROLE SEMANAL AMAZON ADS — WINNET METAIS</t>
   </si>
@@ -172,6 +172,15 @@
   <si>
     <t>06/10/2026 a 12/10/2026</t>
   </si>
+  <si>
+    <t>13/10/2026 a 19/10/2026</t>
+  </si>
+  <si>
+    <t>1ª semana pós-O7 (lances +20%). Entrega −34% e conversão da Geral 0,9% (1 venda em 106 cli); catálogo vendeu só 3 pedidos (R$ 862) — queda de demanda. Sem ação; checkpoint 22/10: Geral ≥150 cli e ≤1 compra → reverter close/substitutes. O8 27/10.</t>
+  </si>
+  <si>
+    <t>relatorios/amazon/monitoramento-19-10/ (export 13–19/10 + print) + ciclos/Monitoramento-19-10.md</t>
+  </si>
 </sst>
 </file>
 
@@ -181,7 +190,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -211,11 +220,6 @@
       <name val="Carlito"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF0F172A"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF475569"/>
@@ -228,14 +232,26 @@
       <name val="Carlito"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <name val="Carlito"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="12"/>
+      <color rgb="FF0F172A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Segoe UI"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -350,14 +366,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -370,9 +383,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -397,24 +407,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -439,9 +431,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -454,26 +443,6 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -483,17 +452,144 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE5E7EB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFECACA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF374151"/>
@@ -588,6 +684,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -672,6 +769,9 @@
                 <c:pt idx="10">
                   <c:v>46307</c:v>
                 </c:pt>
+                <c:pt idx="11">
+                  <c:v>46314</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -715,7 +815,7 @@
                   <c:v>8.3921738671854401E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.7622786759045419</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -860,11 +960,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1962862624"/>
-        <c:axId val="1962858816"/>
+        <c:axId val="-1501044112"/>
+        <c:axId val="-1501039760"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1962862624"/>
+        <c:axId val="-1501044112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -884,7 +984,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1962858816"/>
+        <c:crossAx val="-1501039760"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -892,7 +992,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1962858816"/>
+        <c:axId val="-1501039760"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -912,7 +1012,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1962862624"/>
+        <c:crossAx val="-1501044112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1212,2177 +1312,2201 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
     </row>
     <row r="2" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
     </row>
     <row r="3" spans="1:16" ht="27.95" customHeight="1">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
     </row>
     <row r="4" spans="1:16" ht="21.95" customHeight="1">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47"/>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="30"/>
     </row>
     <row r="5" spans="1:16" ht="33.950000000000003" customHeight="1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="L5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="5" t="s">
+      <c r="P5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
-      <c r="A6" s="28">
+    <row r="6" spans="1:16" ht="15">
+      <c r="A6" s="31">
         <v>46225</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="10">
+      <c r="B6" s="32"/>
+      <c r="C6" s="33">
         <v>32090</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="33">
         <v>140</v>
       </c>
-      <c r="E6" s="33">
+      <c r="E6" s="34">
         <v>128.79</v>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="34">
         <v>371.43</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="35">
         <v>2</v>
       </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="12">
+      <c r="H6" s="35"/>
+      <c r="I6" s="36">
         <f t="shared" ref="I6:I37" si="0">IF(E6=0,"",F6/E6)</f>
         <v>2.883997204751922</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="37">
         <f t="shared" ref="J6:J37" si="1">IF(F6=0,"",E6/F6)</f>
         <v>0.34674097407317661</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="37">
         <f t="shared" ref="K6:K37" si="2">IF(D6=0,"",G6/D6)</f>
         <v>1.4285714285714285E-2</v>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="36">
         <f t="shared" ref="L6:L37" si="3">IF(D6=0,"",E6/D6)</f>
         <v>0.91992857142857132</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="38">
         <f t="shared" ref="M6:M37" si="4">IF(C6=0,"",D6/C6)</f>
         <v>4.3627298223745713E-3</v>
       </c>
-      <c r="N6" s="15"/>
-      <c r="O6" s="1" t="s">
+      <c r="N6" s="32"/>
+      <c r="O6" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="6" t="s">
+      <c r="P6" s="39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
-      <c r="A7" s="28">
+    <row r="7" spans="1:16" ht="15">
+      <c r="A7" s="31">
         <v>46231</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="10">
+      <c r="B7" s="32"/>
+      <c r="C7" s="33">
         <v>20325</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="33">
         <v>110</v>
       </c>
-      <c r="E7" s="33">
+      <c r="E7" s="34">
         <v>70.81</v>
       </c>
-      <c r="F7" s="33">
+      <c r="F7" s="34">
         <v>543.85</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="35">
         <v>1</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="12">
+      <c r="H7" s="35"/>
+      <c r="I7" s="36">
         <f t="shared" si="0"/>
         <v>7.6804123711340209</v>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="37">
         <f t="shared" si="1"/>
         <v>0.13020134228187918</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="37">
         <f t="shared" si="2"/>
         <v>9.0909090909090905E-3</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="36">
         <f t="shared" si="3"/>
         <v>0.6437272727272727</v>
       </c>
-      <c r="M7" s="14">
+      <c r="M7" s="38">
         <f t="shared" si="4"/>
         <v>5.4120541205412058E-3</v>
       </c>
-      <c r="N7" s="15"/>
-      <c r="O7" s="1" t="s">
+      <c r="N7" s="32"/>
+      <c r="O7" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="P7" s="39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="28">
+    <row r="8" spans="1:16" ht="15">
+      <c r="A8" s="31">
         <v>46244</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="10">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33">
         <v>30062</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="33">
         <v>145</v>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="34">
         <v>102.88</v>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="34">
         <v>398.7</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="35">
         <v>2</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="12">
+      <c r="H8" s="35"/>
+      <c r="I8" s="36">
         <f t="shared" si="0"/>
         <v>3.8753888024883358</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="37">
         <f t="shared" si="1"/>
         <v>0.25803862553298218</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="37">
         <f t="shared" si="2"/>
         <v>1.3793103448275862E-2</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="36">
         <f t="shared" si="3"/>
         <v>0.70951724137931027</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="38">
         <f t="shared" si="4"/>
         <v>4.8233650455724838E-3</v>
       </c>
-      <c r="N8" s="15"/>
-      <c r="O8" s="1" t="s">
+      <c r="N8" s="32"/>
+      <c r="O8" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" s="39" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="28.5">
-      <c r="A9" s="30">
+    <row r="9" spans="1:16" ht="15">
+      <c r="A9" s="40">
         <v>46251</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="42">
         <v>16807</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="42">
         <v>102</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="43">
         <v>63.66</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="43">
         <v>132.9</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="44">
         <v>1</v>
       </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="18">
+      <c r="H9" s="44"/>
+      <c r="I9" s="43">
         <f t="shared" si="0"/>
         <v>2.0876531573986807</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="45">
         <f t="shared" si="1"/>
         <v>0.4790067720090293</v>
       </c>
-      <c r="K9" s="19">
+      <c r="K9" s="45">
         <f t="shared" si="2"/>
         <v>9.8039215686274508E-3</v>
       </c>
-      <c r="L9" s="18">
+      <c r="L9" s="43">
         <f t="shared" si="3"/>
         <v>0.62411764705882344</v>
       </c>
-      <c r="M9" s="20">
+      <c r="M9" s="46">
         <f t="shared" si="4"/>
         <v>6.068899863152258E-3</v>
       </c>
-      <c r="N9" s="21"/>
-      <c r="O9" s="2" t="s">
+      <c r="N9" s="41"/>
+      <c r="O9" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="P9" s="7"/>
-    </row>
-    <row r="10" spans="1:16">
-      <c r="A10" s="28">
+      <c r="P9" s="47"/>
+    </row>
+    <row r="10" spans="1:16" ht="15">
+      <c r="A10" s="31">
         <v>46258</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="33">
         <v>36117</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="33">
         <v>127</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="34">
         <v>87.8</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="34">
         <v>2077.2399999999998</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="35">
         <v>2</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="12">
+      <c r="H10" s="35"/>
+      <c r="I10" s="36">
         <f t="shared" si="0"/>
         <v>23.658769931662867</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="37">
         <f t="shared" si="1"/>
         <v>4.2267624347692136E-2</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="37">
         <f t="shared" si="2"/>
         <v>1.5748031496062992E-2</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="36">
         <f t="shared" si="3"/>
         <v>0.6913385826771653</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="38">
         <f t="shared" si="4"/>
         <v>3.5163496414430877E-3</v>
       </c>
-      <c r="N10" s="15" t="s">
+      <c r="N10" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="O10" s="35" t="s">
+      <c r="O10" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="P10" s="6"/>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="A11" s="28">
+      <c r="P10" s="39"/>
+    </row>
+    <row r="11" spans="1:16" ht="15">
+      <c r="A11" s="31">
         <v>46265</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="49">
         <v>47770</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="48">
         <v>197</v>
       </c>
-      <c r="E11" s="39">
+      <c r="E11" s="48">
         <v>156.66</v>
       </c>
-      <c r="F11" s="37">
+      <c r="F11" s="48">
         <v>336.44</v>
       </c>
-      <c r="G11" s="39">
+      <c r="G11" s="48">
         <v>2</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="35">
         <v>2</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="36">
         <f t="shared" si="0"/>
         <v>2.1475807481169413</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="37">
         <f t="shared" si="1"/>
         <v>0.46564023302817736</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="37">
         <f t="shared" si="2"/>
         <v>1.015228426395939E-2</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="36">
         <f t="shared" si="3"/>
         <v>0.79522842639593905</v>
       </c>
-      <c r="M11" s="14">
+      <c r="M11" s="38">
         <f t="shared" si="4"/>
         <v>4.1239271509315471E-3</v>
       </c>
-      <c r="N11" s="15" t="s">
+      <c r="N11" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O11" t="s">
+      <c r="O11" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="P11" t="s">
+      <c r="P11" s="48" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
-      <c r="A12" s="40">
+    <row r="12" spans="1:16" ht="15">
+      <c r="A12" s="50">
         <v>46279</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="33">
         <v>22192</v>
       </c>
-      <c r="D12" s="39">
+      <c r="D12" s="48">
         <v>123</v>
       </c>
-      <c r="E12" s="39">
+      <c r="E12" s="48">
         <v>92.67</v>
       </c>
-      <c r="F12" s="39">
+      <c r="F12" s="48">
         <v>1594.56</v>
       </c>
-      <c r="G12" s="39">
+      <c r="G12" s="48">
         <v>5</v>
       </c>
-      <c r="H12" s="39">
+      <c r="H12" s="48">
         <v>8</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="36">
         <f t="shared" si="0"/>
         <v>17.206863062479766</v>
       </c>
-      <c r="J12" s="13">
+      <c r="J12" s="37">
         <f t="shared" si="1"/>
         <v>5.8116345574954847E-2</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="37">
         <f t="shared" si="2"/>
         <v>4.065040650406504E-2</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="36">
         <f t="shared" si="3"/>
         <v>0.75341463414634147</v>
       </c>
-      <c r="M12" s="14">
+      <c r="M12" s="38">
         <f t="shared" si="4"/>
         <v>5.5425378514780098E-3</v>
       </c>
-      <c r="N12" s="15" t="s">
+      <c r="N12" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O12" s="41" t="s">
+      <c r="O12" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="P12" t="s">
+      <c r="P12" s="48" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
-      <c r="A13" s="28">
+    <row r="13" spans="1:16" ht="15">
+      <c r="A13" s="31">
         <v>46286</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="33">
         <v>43599</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="33">
         <v>146</v>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="34">
         <v>130.55000000000001</v>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="34">
         <v>749.08</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="35">
         <v>2</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="35">
         <v>2</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="36">
         <f t="shared" si="0"/>
         <v>5.737878207583301</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="37">
         <f t="shared" si="1"/>
         <v>0.17428045068617504</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="37">
         <f t="shared" si="2"/>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="36">
         <f t="shared" si="3"/>
         <v>0.89417808219178085</v>
       </c>
-      <c r="M13" s="14">
+      <c r="M13" s="38">
         <f t="shared" si="4"/>
         <v>3.3487006582719786E-3</v>
       </c>
-      <c r="N13" s="15" t="s">
+      <c r="N13" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O13" s="35" t="s">
+      <c r="O13" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="P13" s="42" t="s">
+      <c r="P13" s="39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
-      <c r="A14" s="28">
+    <row r="14" spans="1:16" ht="15">
+      <c r="A14" s="31">
         <v>46293</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="33">
         <v>19379</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="33">
         <v>107</v>
       </c>
-      <c r="E14" s="33">
+      <c r="E14" s="34">
         <v>65.97</v>
       </c>
-      <c r="F14" s="33">
+      <c r="F14" s="34">
         <v>690.28</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="35">
         <v>2</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="35">
         <v>4</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="36">
         <f t="shared" si="0"/>
         <v>10.4635440351675</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="37">
         <f t="shared" si="1"/>
         <v>9.5569913658225647E-2</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="37">
         <f t="shared" si="2"/>
         <v>1.8691588785046728E-2</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="36">
         <f t="shared" si="3"/>
         <v>0.61654205607476631</v>
       </c>
-      <c r="M14" s="14">
+      <c r="M14" s="38">
         <f t="shared" si="4"/>
         <v>5.5214407348160377E-3</v>
       </c>
-      <c r="N14" s="15" t="s">
+      <c r="N14" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="35" t="s">
+      <c r="O14" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P14" s="42" t="s">
+      <c r="P14" s="39" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
-      <c r="A15" s="28">
+    <row r="15" spans="1:16" ht="15">
+      <c r="A15" s="31">
         <v>46300</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="33">
         <v>39236</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="33">
         <v>125</v>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="34">
         <v>110.44</v>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="34">
         <v>3573.64</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="35">
         <v>6</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="35">
         <v>9</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="36">
         <f t="shared" si="0"/>
         <v>32.358203549438606</v>
       </c>
-      <c r="J15" s="13">
+      <c r="J15" s="37">
         <f t="shared" si="1"/>
         <v>3.0904064203445228E-2</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="37">
         <f t="shared" si="2"/>
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="36">
         <f t="shared" si="3"/>
         <v>0.88351999999999997</v>
       </c>
-      <c r="M15" s="14">
+      <c r="M15" s="38">
         <f t="shared" si="4"/>
         <v>3.185849729839943E-3</v>
       </c>
-      <c r="N15" s="15" t="s">
+      <c r="N15" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O15" s="35" t="s">
+      <c r="O15" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="P15" s="42" t="s">
+      <c r="P15" s="39" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="28">
+    <row r="16" spans="1:16" ht="15">
+      <c r="A16" s="31">
         <v>46307</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="33">
         <v>39389</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="33">
         <v>189</v>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="34">
         <v>143.22</v>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="34">
         <v>1706.59</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="35">
         <v>7</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="35">
         <v>12</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="36">
         <f t="shared" si="0"/>
         <v>11.915863706186286</v>
       </c>
-      <c r="J16" s="13">
+      <c r="J16" s="37">
         <f t="shared" si="1"/>
         <v>8.3921738671854401E-2</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="37">
         <f t="shared" si="2"/>
         <v>3.7037037037037035E-2</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="36">
         <f t="shared" si="3"/>
         <v>0.75777777777777777</v>
       </c>
-      <c r="M16" s="14">
+      <c r="M16" s="38">
         <f t="shared" si="4"/>
         <v>4.7982939399324681E-3</v>
       </c>
-      <c r="N16" s="15"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="6"/>
-    </row>
-    <row r="17" spans="1:16">
-      <c r="A17" s="28"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="12" t="str">
+      <c r="N16" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="O16" s="32"/>
+      <c r="P16" s="39"/>
+    </row>
+    <row r="17" spans="1:16" ht="15">
+      <c r="A17" s="31">
+        <v>46314</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="33">
+        <v>25000</v>
+      </c>
+      <c r="D17" s="33">
+        <v>125</v>
+      </c>
+      <c r="E17" s="34">
+        <v>99.02</v>
+      </c>
+      <c r="F17" s="34">
+        <v>129.9</v>
+      </c>
+      <c r="G17" s="35">
+        <v>1</v>
+      </c>
+      <c r="H17" s="35">
+        <v>1</v>
+      </c>
+      <c r="I17" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="13" t="str">
+        <v>1.311856190668552</v>
+      </c>
+      <c r="J17" s="37">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="13" t="str">
+        <v>0.7622786759045419</v>
+      </c>
+      <c r="K17" s="37">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L17" s="12" t="str">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="L17" s="36">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="M17" s="14" t="str">
+        <v>0.79215999999999998</v>
+      </c>
+      <c r="M17" s="38">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="N17" s="15"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="6"/>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="N17" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="O17" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="P17" s="39" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="18" spans="1:16">
-      <c r="A18" s="28"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="12" t="str">
+      <c r="A18" s="20"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J18" s="13" t="str">
+      <c r="J18" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K18" s="13" t="str">
+      <c r="K18" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L18" s="12" t="str">
+      <c r="L18" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M18" s="14" t="str">
+      <c r="M18" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N18" s="15"/>
+      <c r="N18" s="13"/>
       <c r="O18" s="1"/>
-      <c r="P18" s="6"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" spans="1:16">
-      <c r="A19" s="28"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="12" t="str">
+      <c r="A19" s="20"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J19" s="13" t="str">
+      <c r="J19" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K19" s="13" t="str">
+      <c r="K19" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L19" s="12" t="str">
+      <c r="L19" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M19" s="14" t="str">
+      <c r="M19" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N19" s="15"/>
+      <c r="N19" s="13"/>
       <c r="O19" s="1"/>
-      <c r="P19" s="6"/>
+      <c r="P19" s="5"/>
     </row>
     <row r="20" spans="1:16">
-      <c r="A20" s="28"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="12" t="str">
+      <c r="A20" s="20"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J20" s="13" t="str">
+      <c r="J20" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K20" s="13" t="str">
+      <c r="K20" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L20" s="12" t="str">
+      <c r="L20" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M20" s="14" t="str">
+      <c r="M20" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N20" s="15"/>
+      <c r="N20" s="13"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="6"/>
+      <c r="P20" s="5"/>
     </row>
     <row r="21" spans="1:16">
-      <c r="A21" s="28"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="12" t="str">
+      <c r="A21" s="20"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J21" s="13" t="str">
+      <c r="J21" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K21" s="13" t="str">
+      <c r="K21" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L21" s="12" t="str">
+      <c r="L21" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M21" s="14" t="str">
+      <c r="M21" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N21" s="15"/>
+      <c r="N21" s="13"/>
       <c r="O21" s="1"/>
-      <c r="P21" s="6"/>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" spans="1:16">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="12" t="str">
+      <c r="A22" s="20"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J22" s="13" t="str">
+      <c r="J22" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K22" s="13" t="str">
+      <c r="K22" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L22" s="12" t="str">
+      <c r="L22" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M22" s="14" t="str">
+      <c r="M22" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N22" s="15"/>
+      <c r="N22" s="13"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="6"/>
+      <c r="P22" s="5"/>
     </row>
     <row r="23" spans="1:16">
-      <c r="A23" s="28"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="12" t="str">
+      <c r="A23" s="20"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J23" s="13" t="str">
+      <c r="J23" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K23" s="13" t="str">
+      <c r="K23" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L23" s="12" t="str">
+      <c r="L23" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M23" s="14" t="str">
+      <c r="M23" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N23" s="15"/>
+      <c r="N23" s="13"/>
       <c r="O23" s="1"/>
-      <c r="P23" s="6"/>
+      <c r="P23" s="5"/>
     </row>
     <row r="24" spans="1:16">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="12" t="str">
+      <c r="A24" s="20"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J24" s="13" t="str">
+      <c r="J24" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K24" s="13" t="str">
+      <c r="K24" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L24" s="12" t="str">
+      <c r="L24" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M24" s="14" t="str">
+      <c r="M24" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N24" s="15"/>
+      <c r="N24" s="13"/>
       <c r="O24" s="1"/>
-      <c r="P24" s="6"/>
+      <c r="P24" s="5"/>
     </row>
     <row r="25" spans="1:16">
-      <c r="A25" s="28"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="12" t="str">
+      <c r="A25" s="20"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J25" s="13" t="str">
+      <c r="J25" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K25" s="13" t="str">
+      <c r="K25" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L25" s="12" t="str">
+      <c r="L25" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M25" s="14" t="str">
+      <c r="M25" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N25" s="15"/>
+      <c r="N25" s="13"/>
       <c r="O25" s="1"/>
-      <c r="P25" s="6"/>
+      <c r="P25" s="5"/>
     </row>
     <row r="26" spans="1:16">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="12" t="str">
+      <c r="A26" s="20"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J26" s="13" t="str">
+      <c r="J26" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K26" s="13" t="str">
+      <c r="K26" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L26" s="12" t="str">
+      <c r="L26" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M26" s="14" t="str">
+      <c r="M26" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N26" s="15"/>
+      <c r="N26" s="13"/>
       <c r="O26" s="1"/>
-      <c r="P26" s="6"/>
+      <c r="P26" s="5"/>
     </row>
     <row r="27" spans="1:16">
-      <c r="A27" s="28"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="12" t="str">
+      <c r="A27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J27" s="13" t="str">
+      <c r="J27" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K27" s="13" t="str">
+      <c r="K27" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L27" s="12" t="str">
+      <c r="L27" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M27" s="14" t="str">
+      <c r="M27" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N27" s="15"/>
+      <c r="N27" s="13"/>
       <c r="O27" s="1"/>
-      <c r="P27" s="6"/>
+      <c r="P27" s="5"/>
     </row>
     <row r="28" spans="1:16">
-      <c r="A28" s="28"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="12" t="str">
+      <c r="A28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J28" s="13" t="str">
+      <c r="J28" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K28" s="13" t="str">
+      <c r="K28" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L28" s="12" t="str">
+      <c r="L28" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M28" s="14" t="str">
+      <c r="M28" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N28" s="15"/>
+      <c r="N28" s="13"/>
       <c r="O28" s="1"/>
-      <c r="P28" s="6"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" spans="1:16">
-      <c r="A29" s="28"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="12" t="str">
+      <c r="A29" s="20"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J29" s="13" t="str">
+      <c r="J29" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K29" s="13" t="str">
+      <c r="K29" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L29" s="12" t="str">
+      <c r="L29" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M29" s="14" t="str">
+      <c r="M29" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N29" s="15"/>
+      <c r="N29" s="13"/>
       <c r="O29" s="1"/>
-      <c r="P29" s="6"/>
+      <c r="P29" s="5"/>
     </row>
     <row r="30" spans="1:16">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="12" t="str">
+      <c r="A30" s="20"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J30" s="13" t="str">
+      <c r="J30" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K30" s="13" t="str">
+      <c r="K30" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L30" s="12" t="str">
+      <c r="L30" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M30" s="14" t="str">
+      <c r="M30" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N30" s="15"/>
+      <c r="N30" s="13"/>
       <c r="O30" s="1"/>
-      <c r="P30" s="6"/>
+      <c r="P30" s="5"/>
     </row>
     <row r="31" spans="1:16">
-      <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="12" t="str">
+      <c r="A31" s="20"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J31" s="13" t="str">
+      <c r="J31" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K31" s="13" t="str">
+      <c r="K31" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L31" s="12" t="str">
+      <c r="L31" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M31" s="14" t="str">
+      <c r="M31" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N31" s="15"/>
+      <c r="N31" s="13"/>
       <c r="O31" s="1"/>
-      <c r="P31" s="6"/>
+      <c r="P31" s="5"/>
     </row>
     <row r="32" spans="1:16">
-      <c r="A32" s="28"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="12" t="str">
+      <c r="A32" s="20"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J32" s="13" t="str">
+      <c r="J32" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K32" s="13" t="str">
+      <c r="K32" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L32" s="12" t="str">
+      <c r="L32" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M32" s="14" t="str">
+      <c r="M32" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N32" s="15"/>
+      <c r="N32" s="13"/>
       <c r="O32" s="1"/>
-      <c r="P32" s="6"/>
+      <c r="P32" s="5"/>
     </row>
     <row r="33" spans="1:16">
-      <c r="A33" s="28"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="12" t="str">
+      <c r="A33" s="20"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J33" s="13" t="str">
+      <c r="J33" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K33" s="13" t="str">
+      <c r="K33" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L33" s="12" t="str">
+      <c r="L33" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M33" s="14" t="str">
+      <c r="M33" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N33" s="15"/>
+      <c r="N33" s="13"/>
       <c r="O33" s="1"/>
-      <c r="P33" s="6"/>
+      <c r="P33" s="5"/>
     </row>
     <row r="34" spans="1:16">
-      <c r="A34" s="28"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="12" t="str">
+      <c r="A34" s="20"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J34" s="13" t="str">
+      <c r="J34" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K34" s="13" t="str">
+      <c r="K34" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L34" s="12" t="str">
+      <c r="L34" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M34" s="14" t="str">
+      <c r="M34" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N34" s="15"/>
+      <c r="N34" s="13"/>
       <c r="O34" s="1"/>
-      <c r="P34" s="6"/>
+      <c r="P34" s="5"/>
     </row>
     <row r="35" spans="1:16">
-      <c r="A35" s="28"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="12" t="str">
+      <c r="A35" s="20"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J35" s="13" t="str">
+      <c r="J35" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K35" s="13" t="str">
+      <c r="K35" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L35" s="12" t="str">
+      <c r="L35" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M35" s="14" t="str">
+      <c r="M35" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N35" s="15"/>
+      <c r="N35" s="13"/>
       <c r="O35" s="1"/>
-      <c r="P35" s="6"/>
+      <c r="P35" s="5"/>
     </row>
     <row r="36" spans="1:16">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="12" t="str">
+      <c r="A36" s="20"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J36" s="13" t="str">
+      <c r="J36" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K36" s="13" t="str">
+      <c r="K36" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L36" s="12" t="str">
+      <c r="L36" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M36" s="14" t="str">
+      <c r="M36" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N36" s="15"/>
+      <c r="N36" s="13"/>
       <c r="O36" s="1"/>
-      <c r="P36" s="6"/>
+      <c r="P36" s="5"/>
     </row>
     <row r="37" spans="1:16">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="12" t="str">
+      <c r="A37" s="20"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J37" s="13" t="str">
+      <c r="J37" s="11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K37" s="13" t="str">
+      <c r="K37" s="11" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L37" s="12" t="str">
+      <c r="L37" s="10" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M37" s="14" t="str">
+      <c r="M37" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N37" s="15"/>
+      <c r="N37" s="13"/>
       <c r="O37" s="1"/>
-      <c r="P37" s="6"/>
+      <c r="P37" s="5"/>
     </row>
     <row r="38" spans="1:16">
-      <c r="A38" s="28"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="12" t="str">
+      <c r="A38" s="20"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="10" t="str">
         <f t="shared" ref="I38:I60" si="5">IF(E38=0,"",F38/E38)</f>
         <v/>
       </c>
-      <c r="J38" s="13" t="str">
+      <c r="J38" s="11" t="str">
         <f t="shared" ref="J38:J60" si="6">IF(F38=0,"",E38/F38)</f>
         <v/>
       </c>
-      <c r="K38" s="13" t="str">
+      <c r="K38" s="11" t="str">
         <f t="shared" ref="K38:K60" si="7">IF(D38=0,"",G38/D38)</f>
         <v/>
       </c>
-      <c r="L38" s="12" t="str">
+      <c r="L38" s="10" t="str">
         <f t="shared" ref="L38:L60" si="8">IF(D38=0,"",E38/D38)</f>
         <v/>
       </c>
-      <c r="M38" s="14" t="str">
+      <c r="M38" s="12" t="str">
         <f t="shared" ref="M38:M60" si="9">IF(C38=0,"",D38/C38)</f>
         <v/>
       </c>
-      <c r="N38" s="15"/>
+      <c r="N38" s="13"/>
       <c r="O38" s="1"/>
-      <c r="P38" s="6"/>
+      <c r="P38" s="5"/>
     </row>
     <row r="39" spans="1:16">
-      <c r="A39" s="28"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="12" t="str">
+      <c r="A39" s="20"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J39" s="13" t="str">
+      <c r="J39" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K39" s="13" t="str">
+      <c r="K39" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L39" s="12" t="str">
+      <c r="L39" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M39" s="14" t="str">
+      <c r="M39" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N39" s="15"/>
+      <c r="N39" s="13"/>
       <c r="O39" s="1"/>
-      <c r="P39" s="6"/>
+      <c r="P39" s="5"/>
     </row>
     <row r="40" spans="1:16">
-      <c r="A40" s="28"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="12" t="str">
+      <c r="A40" s="20"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J40" s="13" t="str">
+      <c r="J40" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K40" s="13" t="str">
+      <c r="K40" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L40" s="12" t="str">
+      <c r="L40" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M40" s="14" t="str">
+      <c r="M40" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N40" s="15"/>
+      <c r="N40" s="13"/>
       <c r="O40" s="1"/>
-      <c r="P40" s="6"/>
+      <c r="P40" s="5"/>
     </row>
     <row r="41" spans="1:16">
-      <c r="A41" s="28"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="12" t="str">
+      <c r="A41" s="20"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J41" s="13" t="str">
+      <c r="J41" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K41" s="13" t="str">
+      <c r="K41" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L41" s="12" t="str">
+      <c r="L41" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M41" s="14" t="str">
+      <c r="M41" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N41" s="15"/>
+      <c r="N41" s="13"/>
       <c r="O41" s="1"/>
-      <c r="P41" s="6"/>
+      <c r="P41" s="5"/>
     </row>
     <row r="42" spans="1:16">
-      <c r="A42" s="28"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="12" t="str">
+      <c r="A42" s="20"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J42" s="13" t="str">
+      <c r="J42" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K42" s="13" t="str">
+      <c r="K42" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L42" s="12" t="str">
+      <c r="L42" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M42" s="14" t="str">
+      <c r="M42" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N42" s="15"/>
+      <c r="N42" s="13"/>
       <c r="O42" s="1"/>
-      <c r="P42" s="6"/>
+      <c r="P42" s="5"/>
     </row>
     <row r="43" spans="1:16">
-      <c r="A43" s="28"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="12" t="str">
+      <c r="A43" s="20"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J43" s="13" t="str">
+      <c r="J43" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K43" s="13" t="str">
+      <c r="K43" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L43" s="12" t="str">
+      <c r="L43" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M43" s="14" t="str">
+      <c r="M43" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N43" s="15"/>
+      <c r="N43" s="13"/>
       <c r="O43" s="1"/>
-      <c r="P43" s="6"/>
+      <c r="P43" s="5"/>
     </row>
     <row r="44" spans="1:16">
-      <c r="A44" s="28"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="12" t="str">
+      <c r="A44" s="20"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J44" s="13" t="str">
+      <c r="J44" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K44" s="13" t="str">
+      <c r="K44" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L44" s="12" t="str">
+      <c r="L44" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M44" s="14" t="str">
+      <c r="M44" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N44" s="15"/>
+      <c r="N44" s="13"/>
       <c r="O44" s="1"/>
-      <c r="P44" s="6"/>
+      <c r="P44" s="5"/>
     </row>
     <row r="45" spans="1:16">
-      <c r="A45" s="28"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="12" t="str">
+      <c r="A45" s="20"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J45" s="13" t="str">
+      <c r="J45" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K45" s="13" t="str">
+      <c r="K45" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L45" s="12" t="str">
+      <c r="L45" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M45" s="14" t="str">
+      <c r="M45" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N45" s="15"/>
+      <c r="N45" s="13"/>
       <c r="O45" s="1"/>
-      <c r="P45" s="6"/>
+      <c r="P45" s="5"/>
     </row>
     <row r="46" spans="1:16">
-      <c r="A46" s="28"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="33"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="11"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="12" t="str">
+      <c r="A46" s="20"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J46" s="13" t="str">
+      <c r="J46" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K46" s="13" t="str">
+      <c r="K46" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L46" s="12" t="str">
+      <c r="L46" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M46" s="14" t="str">
+      <c r="M46" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N46" s="15"/>
+      <c r="N46" s="13"/>
       <c r="O46" s="1"/>
-      <c r="P46" s="6"/>
+      <c r="P46" s="5"/>
     </row>
     <row r="47" spans="1:16">
-      <c r="A47" s="28"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="33"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="12" t="str">
+      <c r="A47" s="20"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J47" s="13" t="str">
+      <c r="J47" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K47" s="13" t="str">
+      <c r="K47" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L47" s="12" t="str">
+      <c r="L47" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M47" s="14" t="str">
+      <c r="M47" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N47" s="15"/>
+      <c r="N47" s="13"/>
       <c r="O47" s="1"/>
-      <c r="P47" s="6"/>
+      <c r="P47" s="5"/>
     </row>
     <row r="48" spans="1:16">
-      <c r="A48" s="28"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="12" t="str">
+      <c r="A48" s="20"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="24"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+      <c r="I48" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J48" s="13" t="str">
+      <c r="J48" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K48" s="13" t="str">
+      <c r="K48" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L48" s="12" t="str">
+      <c r="L48" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M48" s="14" t="str">
+      <c r="M48" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N48" s="15"/>
+      <c r="N48" s="13"/>
       <c r="O48" s="1"/>
-      <c r="P48" s="6"/>
+      <c r="P48" s="5"/>
     </row>
     <row r="49" spans="1:16">
-      <c r="A49" s="28"/>
-      <c r="B49" s="29"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="12" t="str">
+      <c r="A49" s="20"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+      <c r="I49" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J49" s="13" t="str">
+      <c r="J49" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K49" s="13" t="str">
+      <c r="K49" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L49" s="12" t="str">
+      <c r="L49" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M49" s="14" t="str">
+      <c r="M49" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N49" s="15"/>
+      <c r="N49" s="13"/>
       <c r="O49" s="1"/>
-      <c r="P49" s="6"/>
+      <c r="P49" s="5"/>
     </row>
     <row r="50" spans="1:16">
-      <c r="A50" s="28"/>
-      <c r="B50" s="29"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="12" t="str">
+      <c r="A50" s="20"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+      <c r="I50" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J50" s="13" t="str">
+      <c r="J50" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K50" s="13" t="str">
+      <c r="K50" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L50" s="12" t="str">
+      <c r="L50" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M50" s="14" t="str">
+      <c r="M50" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N50" s="15"/>
+      <c r="N50" s="13"/>
       <c r="O50" s="1"/>
-      <c r="P50" s="6"/>
+      <c r="P50" s="5"/>
     </row>
     <row r="51" spans="1:16">
-      <c r="A51" s="28"/>
-      <c r="B51" s="29"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="11"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="12" t="str">
+      <c r="A51" s="20"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J51" s="13" t="str">
+      <c r="J51" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K51" s="13" t="str">
+      <c r="K51" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L51" s="12" t="str">
+      <c r="L51" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M51" s="14" t="str">
+      <c r="M51" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N51" s="15"/>
+      <c r="N51" s="13"/>
       <c r="O51" s="1"/>
-      <c r="P51" s="6"/>
+      <c r="P51" s="5"/>
     </row>
     <row r="52" spans="1:16">
-      <c r="A52" s="28"/>
-      <c r="B52" s="29"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="11"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="12" t="str">
+      <c r="A52" s="20"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+      <c r="I52" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J52" s="13" t="str">
+      <c r="J52" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K52" s="13" t="str">
+      <c r="K52" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L52" s="12" t="str">
+      <c r="L52" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M52" s="14" t="str">
+      <c r="M52" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N52" s="15"/>
+      <c r="N52" s="13"/>
       <c r="O52" s="1"/>
-      <c r="P52" s="6"/>
+      <c r="P52" s="5"/>
     </row>
     <row r="53" spans="1:16">
-      <c r="A53" s="28"/>
-      <c r="B53" s="29"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
-      <c r="G53" s="11"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="12" t="str">
+      <c r="A53" s="20"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J53" s="13" t="str">
+      <c r="J53" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K53" s="13" t="str">
+      <c r="K53" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L53" s="12" t="str">
+      <c r="L53" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M53" s="14" t="str">
+      <c r="M53" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N53" s="15"/>
+      <c r="N53" s="13"/>
       <c r="O53" s="1"/>
-      <c r="P53" s="6"/>
+      <c r="P53" s="5"/>
     </row>
     <row r="54" spans="1:16">
-      <c r="A54" s="28"/>
-      <c r="B54" s="29"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="33"/>
-      <c r="F54" s="33"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="12" t="str">
+      <c r="A54" s="20"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J54" s="13" t="str">
+      <c r="J54" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K54" s="13" t="str">
+      <c r="K54" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L54" s="12" t="str">
+      <c r="L54" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M54" s="14" t="str">
+      <c r="M54" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N54" s="15"/>
+      <c r="N54" s="13"/>
       <c r="O54" s="1"/>
-      <c r="P54" s="6"/>
+      <c r="P54" s="5"/>
     </row>
     <row r="55" spans="1:16">
-      <c r="A55" s="28"/>
-      <c r="B55" s="29"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="33"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="12" t="str">
+      <c r="A55" s="20"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J55" s="13" t="str">
+      <c r="J55" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K55" s="13" t="str">
+      <c r="K55" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L55" s="12" t="str">
+      <c r="L55" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M55" s="14" t="str">
+      <c r="M55" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N55" s="15"/>
+      <c r="N55" s="13"/>
       <c r="O55" s="1"/>
-      <c r="P55" s="6"/>
+      <c r="P55" s="5"/>
     </row>
     <row r="56" spans="1:16">
-      <c r="A56" s="28"/>
-      <c r="B56" s="29"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="12" t="str">
+      <c r="A56" s="20"/>
+      <c r="B56" s="21"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="24"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J56" s="13" t="str">
+      <c r="J56" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K56" s="13" t="str">
+      <c r="K56" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L56" s="12" t="str">
+      <c r="L56" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M56" s="14" t="str">
+      <c r="M56" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N56" s="15"/>
+      <c r="N56" s="13"/>
       <c r="O56" s="1"/>
-      <c r="P56" s="6"/>
+      <c r="P56" s="5"/>
     </row>
     <row r="57" spans="1:16">
-      <c r="A57" s="28"/>
-      <c r="B57" s="29"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="33"/>
-      <c r="F57" s="33"/>
-      <c r="G57" s="11"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="12" t="str">
+      <c r="A57" s="20"/>
+      <c r="B57" s="21"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="24"/>
+      <c r="F57" s="24"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
+      <c r="I57" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J57" s="13" t="str">
+      <c r="J57" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K57" s="13" t="str">
+      <c r="K57" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L57" s="12" t="str">
+      <c r="L57" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M57" s="14" t="str">
+      <c r="M57" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N57" s="15"/>
+      <c r="N57" s="13"/>
       <c r="O57" s="1"/>
-      <c r="P57" s="6"/>
+      <c r="P57" s="5"/>
     </row>
     <row r="58" spans="1:16">
-      <c r="A58" s="28"/>
-      <c r="B58" s="29"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="33"/>
-      <c r="F58" s="33"/>
-      <c r="G58" s="11"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="12" t="str">
+      <c r="A58" s="20"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J58" s="13" t="str">
+      <c r="J58" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K58" s="13" t="str">
+      <c r="K58" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L58" s="12" t="str">
+      <c r="L58" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M58" s="14" t="str">
+      <c r="M58" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N58" s="15"/>
+      <c r="N58" s="13"/>
       <c r="O58" s="1"/>
-      <c r="P58" s="6"/>
+      <c r="P58" s="5"/>
     </row>
     <row r="59" spans="1:16">
-      <c r="A59" s="28"/>
-      <c r="B59" s="29"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
-      <c r="G59" s="11"/>
-      <c r="H59" s="11"/>
-      <c r="I59" s="12" t="str">
+      <c r="A59" s="20"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="10" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J59" s="13" t="str">
+      <c r="J59" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K59" s="13" t="str">
+      <c r="K59" s="11" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L59" s="12" t="str">
+      <c r="L59" s="10" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M59" s="14" t="str">
+      <c r="M59" s="12" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N59" s="15"/>
+      <c r="N59" s="13"/>
       <c r="O59" s="1"/>
-      <c r="P59" s="6"/>
+      <c r="P59" s="5"/>
     </row>
     <row r="60" spans="1:16">
-      <c r="A60" s="31"/>
-      <c r="B60" s="32"/>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="23"/>
-      <c r="H60" s="23"/>
-      <c r="I60" s="24" t="str">
+      <c r="A60" s="22"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="25"/>
+      <c r="F60" s="25"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="16" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J60" s="25" t="str">
+      <c r="J60" s="17" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K60" s="25" t="str">
+      <c r="K60" s="17" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L60" s="24" t="str">
+      <c r="L60" s="16" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M60" s="26" t="str">
+      <c r="M60" s="18" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="N60" s="27"/>
-      <c r="O60" s="8"/>
-      <c r="P60" s="9"/>
+      <c r="N60" s="19"/>
+      <c r="O60" s="6"/>
+      <c r="P60" s="7"/>
     </row>
     <row r="62" spans="1:16" ht="26.1" customHeight="1">
-      <c r="A62" s="46" t="s">
+      <c r="A62" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="46"/>
-      <c r="C62" s="46"/>
-      <c r="D62" s="46"/>
-      <c r="E62" s="46"/>
-      <c r="F62" s="46"/>
-      <c r="G62" s="46"/>
-      <c r="H62" s="46"/>
-      <c r="I62" s="46"/>
-      <c r="J62" s="46"/>
-      <c r="K62" s="46"/>
-      <c r="L62" s="46"/>
-      <c r="M62" s="46"/>
-      <c r="N62" s="46"/>
-      <c r="O62" s="46"/>
-      <c r="P62" s="46"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="29"/>
+      <c r="E62" s="29"/>
+      <c r="F62" s="29"/>
+      <c r="G62" s="29"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="29"/>
+      <c r="J62" s="29"/>
+      <c r="K62" s="29"/>
+      <c r="L62" s="29"/>
+      <c r="M62" s="29"/>
+      <c r="N62" s="29"/>
+      <c r="O62" s="29"/>
+      <c r="P62" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3393,22 +3517,22 @@
     <mergeCell ref="A4:P4"/>
   </mergeCells>
   <conditionalFormatting sqref="N6:N60">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>N6="NORMAL / AGUARDAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>N6="VIGIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>N6="INVESTIGAR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>N6="PROBLEMA OPERACIONAL"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>N6="EMERGÊNCIA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>N6="DADO INSUFICIENTE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>